<commit_message>
database rework and backend changes
</commit_message>
<xml_diff>
--- a/docs/Anforderungskatalog_16092026.xlsx
+++ b/docs/Anforderungskatalog_16092026.xlsx
@@ -414,7 +414,7 @@
     </row>
     <row r="2" ht="28" customHeight="1">
       <c r="A2" s="12" t="str">
-        <v>Fachstand 18.09.2026 mit freigegebenen Revisionen bis 21.09.2026; 54 aktive Anforderungen, keine neuen IDs</v>
+        <v>Fachstand 18.09.2026 mit freigegebenen Revisionen bis 24.09.2026; 54 aktive Anforderungen, keine neuen IDs</v>
       </c>
       <c r="B2" s="12"/>
       <c r="C2" s="12"/>
@@ -492,13 +492,13 @@
       <c r="D9" s="16"/>
       <c r="E9" s="16"/>
     </row>
-    <row r="10" ht="44" customHeight="1">
+    <row r="10" ht="150" customHeight="1">
       <c r="A10" s="17"/>
       <c r="B10" s="17" t="str">
         <v>G-06</v>
       </c>
       <c r="C10" s="17" t="str">
-        <v>Jeder Mitarbeiter wird genau einer Organisationseinheit zugeordnet; eine gleichzeitige Zuordnung zu mehreren Organisationseinheiten ist ausgeschlossen.</v>
+        <v>Mitarbeitende und Aufgaben werden Organisationseinheiten über m:n-Zuordnungen zugeordnet. Derselbe Mitarbeiter und dieselbe Aufgabe können mehreren Einheiten angehören, ohne ihre Stammdatensätze zu duplizieren. Vorher- und Nachher-Stände werden als getrennte vorbereitete Organisationseinheiten betrachtet. Direkte Mitarbeiter-Skills werden je Organisationszuordnung separat gespeichert; derselbe Skill darf für dieselbe Person in mehreren Einheiten vorkommen, innerhalb einer Einheit jedoch nur einmal. Skillzuordnungen setzen eine gültige Organisationszuordnung der Person voraus.</v>
       </c>
       <c r="D10" s="17"/>
       <c r="E10" s="17"/>
@@ -567,13 +567,13 @@
       <c r="D16" s="16"/>
       <c r="E16" s="16"/>
     </row>
-    <row r="17" ht="150" customHeight="1">
+    <row r="17" ht="105" customHeight="1">
       <c r="A17" s="17"/>
       <c r="B17" s="17" t="str">
         <v>G-05</v>
       </c>
       <c r="C17" s="17" t="str">
-        <v>Das Webinterface sollte eine funktionsfähige Auswahl der in der Datenbank vorhandenen Organisationseinheiten anbieten. Ein Wechsel lädt ausschließlich die Aufgaben und Mitarbeitenden der gewählten Einheit und setzt Simulation, Masken, Navigation, Ansicht und Distanzgrenze auf den Ausgangszustand zurück. Daraus entsteht keine Verwaltungsfunktion.</v>
+        <v>Das Webinterface sollte eine funktionsfähige Auswahl der in der Datenbank vorhandenen Organisationseinheiten anbieten. Ein Wechsel lädt ausschließlich die zugeordneten Aufgaben und Mitarbeitenden sowie die für diese Einheit gespeicherten Mitarbeiter-Skills und setzt Simulation, Masken, Navigation, Ansicht und Distanzgrenze auf den Ausgangszustand zurück. Daraus entsteht keine Verwaltungsfunktion.</v>
       </c>
       <c r="D17" s="17"/>
       <c r="E17" s="17"/>
@@ -627,24 +627,24 @@
       <c r="D22" s="17"/>
       <c r="E22" s="17"/>
     </row>
-    <row r="23" ht="60" customHeight="1">
+    <row r="23" ht="105" customHeight="1">
       <c r="A23" s="17"/>
       <c r="B23" s="17" t="str">
         <v>D-07</v>
       </c>
       <c r="C23" s="17" t="str">
-        <v>Für jede eingeschlossene Aufgabe müssen ihre direkt zugeordneten Skills und sämtliche eindeutigen direkten und indirekten Voraussetzungen als benötigt gelten. Die impliziten Zuordnungen werden bei der Auswertung hergeleitet und nicht zusätzlich dauerhaft gespeichert.</v>
+        <v>Für jede eingeschlossene Aufgabe müssen ihre direkt zugeordneten Skills und sämtliche eindeutigen direkten und indirekten Voraussetzungen als benötigt gelten. Die direkten Skillanforderungen einer Aufgabe gelten in allen zugeordneten Organisationseinheiten identisch. Die impliziten Zuordnungen werden bei der Auswertung hergeleitet und nicht zusätzlich dauerhaft gespeichert.</v>
       </c>
       <c r="D23" s="17"/>
       <c r="E23" s="17"/>
     </row>
-    <row r="24" ht="60" customHeight="1">
+    <row r="24" ht="105" customHeight="1">
       <c r="A24" s="17"/>
       <c r="B24" s="17" t="str">
         <v>D-08</v>
       </c>
       <c r="C24" s="17" t="str">
-        <v>Für jeden Mitarbeiter müssen seine direkt zugeordneten Skills und sämtliche eindeutigen direkten und indirekten Voraussetzungen als vorhanden gelten. Die impliziten Zuordnungen werden bei der Auswertung hergeleitet und nicht zusätzlich dauerhaft gespeichert.</v>
+        <v>Für jeden eingeschlossenen Mitarbeiter müssen ausschließlich seine in der ausgewählten Organisationseinheit direkt zugeordneten Skills und sämtliche eindeutigen direkten und indirekten Voraussetzungen als vorhanden gelten. Skillzuordnungen derselben Person in anderen Einheiten werden nicht übernommen. Die impliziten Zuordnungen werden bei der Auswertung hergeleitet und nicht zusätzlich dauerhaft gespeichert.</v>
       </c>
       <c r="D24" s="17"/>
       <c r="E24" s="17"/>

</xml_diff>

<commit_message>
Addition: Skill <> Task Assignment in the UI
</commit_message>
<xml_diff>
--- a/docs/Anforderungskatalog_16092026.xlsx
+++ b/docs/Anforderungskatalog_16092026.xlsx
@@ -414,7 +414,7 @@
     </row>
     <row r="2" ht="28" customHeight="1">
       <c r="A2" s="12" t="str">
-        <v>Fachstand 18.09.2026 mit freigegebenen Revisionen bis 24.09.2026; 54 aktive Anforderungen, keine neuen IDs</v>
+        <v>Fachstand 18.09.2026 mit freigegebenen Revisionen bis 25.09.2026; 54 aktive Anforderungen, keine neuen IDs</v>
       </c>
       <c r="B2" s="12"/>
       <c r="C2" s="12"/>
@@ -1102,13 +1102,13 @@
       <c r="D67" s="17"/>
       <c r="E67" s="17"/>
     </row>
-    <row r="68" ht="76" customHeight="1">
+    <row r="68" ht="210" customHeight="1">
       <c r="A68" s="17"/>
       <c r="B68" s="17" t="str">
         <v>S-04</v>
       </c>
       <c r="C68" s="17" t="str">
-        <v>Die Auswahl eines Kandidaten aus einer Handlungsempfehlung oder der Aufruf eines Skills mit ausgewählter Person muss den personenbezogenen verbleibenden Entwicklungspfad zum Zielskill öffnen, sofern der Skill gemäß S-01 geschätzt ist. In der Pfadansicht muss der Personenbezug gewechselt oder über Allgemein aufgehoben werden können.</v>
+        <v>Die Auswahl eines Kandidaten aus einer Handlungsempfehlung oder der Aufruf eines Skills mit ausgewählter Person muss den personenbezogenen verbleibenden Entwicklungspfad zum Zielskill öffnen, sofern der Skill gemäß S-01 geschätzt ist. In der Pfadansicht muss der Personenbezug gewechselt oder über Allgemein aufgehoben werden können. Die personenbezogene Pfadansicht bietet dieselbe zielskillbezogene Aufgabenzuordnung wie die allgemeine Ansicht gemäß S-07; Personenauswahl und Pfadumfang verändern diese Liste nicht.</v>
       </c>
       <c r="D68" s="17"/>
       <c r="E68" s="17"/>
@@ -1135,13 +1135,13 @@
       <c r="D70" s="17"/>
       <c r="E70" s="17"/>
     </row>
-    <row r="71" ht="60" customHeight="1">
+    <row r="71" ht="255" customHeight="1">
       <c r="A71" s="17"/>
       <c r="B71" s="17" t="str">
         <v>S-07</v>
       </c>
       <c r="C71" s="17" t="str">
-        <v>Ein Skillaufruf ohne ausgewählte Person muss bei Verfügbarkeit gemäß S-01 den vollständigen allgemeinen DAG ohne personenbezogene Besitzbewertung öffnen. Die Organisationsmaske darf keine Voraussetzungen aus Berechnung oder fachlichem Umfang des gewählten DAGs entfernen.</v>
+        <v>Ein Skillaufruf ohne ausgewählte Person muss bei Verfügbarkeit gemäß S-01 den vollständigen allgemeinen DAG ohne personenbezogene Besitzbewertung öffnen. Die Organisationsmaske darf keine Voraussetzungen aus Berechnung oder fachlichem Umfang des gewählten DAGs entfernen. Der Knopf „Aufgabenzuordnung“ öffnet ein modales Popup mit den Aufgaben, die genau den Zielskill direkt oder als direkte beziehungsweise indirekte Voraussetzung ihrer zugeordneten Skills benötigen, ausschließlich innerhalb der ausgewählten Organisationseinheit. Jede Aufgabe erscheint einmal, auch bei mehreren Vererbungswegen. Temporär ausgeschlossene Aufgaben bleiben mit dem Hinweis „in Simulation ausgeschlossen“ sichtbar. Die Anzeige lautet „Aufgabe [ID] • [Aufgabenname]“; bei leerem Namen steht „kein Aufgabenname hinterlegt“. Ohne Zuordnung erscheint ein Leerhinweis. Der Inhalt ist bei Überlänge scrollbar; Überschrift und Schließen-Knopf bleiben sichtbar. Schließen erhält Ansicht, Auswahl und Scrollposition.</v>
       </c>
       <c r="D71" s="17"/>
       <c r="E71" s="17"/>

</xml_diff>